<commit_message>
add clear screen function
</commit_message>
<xml_diff>
--- a/READING/2_22_12.xlsx
+++ b/READING/2_22_12.xlsx
@@ -492,16 +492,16 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>できるだけ</t>
+          <t>たいてい</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>尽可能地，尽量</t>
+          <t>大抵，大都</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -510,38 +510,34 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>持ち歩く</t>
+          <t>により</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>携带；随身携带</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>もちあるく</t>
-        </is>
-      </c>
+          <t>根据，由于</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>立ち寄る</t>
+          <t>および</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>顺路去；顺便到</t>
+          <t>以及，和</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -550,7 +546,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -572,25 +568,29 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>すでに</t>
+          <t>ほしがる</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>已经</t>
+          <t>（第三方）想要</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>たがる-&gt;第三人称想要</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -634,34 +634,38 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ほうっておく</t>
+          <t>直後</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>置之不理，放任不管</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
+          <t>之后不久，紧接着</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ちょくご</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>だいぶ</t>
+          <t>なぐさめる</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>相当；颇；很；很多</t>
+          <t>安慰，慰问</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -670,38 +674,38 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>真剣さ</t>
+          <t>いっこう〜ない</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>认真，严肃（的程度）</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>しんけんさ</t>
-        </is>
-      </c>
+          <t>一点也（不）......</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>まったく-&gt;完全地</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>それだけ</t>
+          <t>それぞれ</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>只有那么些，仅此而已</t>
+          <t>各自，分别</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -714,37 +718,41 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>なくす</t>
+          <t>〜方がいい</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>弄丢，失去</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
+          <t>最好…</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>〜ほうがいい</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>とれる</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>それぞれ</t>
+          <t>生産的</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>各自，分别</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+          <t>有生产性的，有成果的</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>せいさんてき</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
     </row>
@@ -754,30 +762,34 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>必ずしも〜ない</t>
+          <t>なくす</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>未必，不一定</t>
+          <t>弄丢，失去</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>とれる</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>たいてい</t>
+          <t>必ずしも〜ない</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>大抵，大都</t>
+          <t>未必，不一定</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -786,38 +798,34 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>いっこう〜ない</t>
+          <t>できるだけ</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>一点也（不）......</t>
+          <t>尽可能地，尽量</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>まったく-&gt;完全地</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>なぐさめる</t>
+          <t>それだけ</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>安慰，慰问</t>
+          <t>只有那么些，仅此而已</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -830,17 +838,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>生産的</t>
+          <t>真剣さ</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>有生产性的，有成果的</t>
+          <t>认真，严肃（的程度）</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>せいさんてき</t>
+          <t>しんけんさ</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -848,82 +856,70 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>直後</t>
+          <t>だいぶ</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>之后不久，紧接着</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>ちょくご</t>
-        </is>
-      </c>
+          <t>相当；颇；很；很多</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>〜方がいい</t>
+          <t>ほうっておく</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>最好…</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>〜ほうがいい</t>
-        </is>
-      </c>
+          <t>置之不理，放任不管</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ほしがる</t>
+          <t>すでに</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>（第三方）想要</t>
+          <t>已经</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>たがる-&gt;第三人称想要</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>および</t>
+          <t>立ち寄る</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>以及，和</t>
+          <t>顺路去；顺便到</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -936,21 +932,25 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>により</t>
+          <t>持ち歩く</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>根据，由于</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
+          <t>携带；随身携带</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>もちあるく</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
2-4 second short reading
</commit_message>
<xml_diff>
--- a/READING/2_22_12.xlsx
+++ b/READING/2_22_12.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\N2_2025_12\READING\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADE9C911-E437-4A5A-B1B8-FD74B62BCF68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13D95A1F-991A-4406-AB98-5F6FDDA9CA7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14820" yWindow="4275" windowWidth="23580" windowHeight="9255" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10560" yWindow="885" windowWidth="27840" windowHeight="20040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
   <si>
     <t>Fre</t>
   </si>
@@ -219,20 +219,157 @@
     <t>顺路去；顺便到</t>
   </si>
   <si>
+    <t>最好…</t>
+  </si>
+  <si>
+    <t>〜ほうがいい</t>
+  </si>
+  <si>
+    <t>あまり～ない</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>不太…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ならば</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>如果…的话</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>採用の面接</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>录用面试</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>由于；通过；根据</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>〜により</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>先</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>地点，目的地；前面；尖端</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>えさ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>饲料；诱饵</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>あまりほしがらなくなります</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>变得不怎么想要</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>で</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>并且</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ておけば</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>モデル</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>款式，模型</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>だけでなく</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>不仅仅</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>すべて</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>全部，所有</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>これほど～ないだろう</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>没有比这更…的吧(最高级)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>もしかしたら</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>或许，说不定</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>順番</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>顺序</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ふつう</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>普通，通常，平常</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ただ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>仅仅；免费</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>〜方がいい</t>
-  </si>
-  <si>
-    <t>最好…</t>
-  </si>
-  <si>
-    <t>〜ほうがいい</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>"ておく"提前</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -241,17 +378,27 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="9"/>
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="2">
@@ -289,11 +436,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -596,7 +744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="2" max="2" width="25.875" customWidth="1"/>
@@ -623,321 +771,579 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A2">
+      <c r="A2" s="2">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A3">
+      <c r="A3" s="2">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E3" t="s">
+      <c r="D3" s="2"/>
+      <c r="E3" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E4" t="s">
+      <c r="D4" s="2"/>
+      <c r="E4" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="A5" s="2">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E5" t="s">
+      <c r="D5" s="2"/>
+      <c r="E5" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A6">
+      <c r="A6" s="2">
         <v>3</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="2" t="s">
         <v>18</v>
       </c>
+      <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A7">
+      <c r="A7" s="2">
         <v>3</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
+      <c r="E7" s="2"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A8">
-        <v>2</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="A8" s="2">
+        <v>2</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>23</v>
       </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A9">
+      <c r="A9" s="2">
         <v>3</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E9" t="s">
+      <c r="D9" s="2"/>
+      <c r="E9" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A10">
+      <c r="A10" s="2">
         <v>1</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E10" t="s">
+      <c r="D10" s="2"/>
+      <c r="E10" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A11">
+      <c r="A11" s="2">
         <v>1</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="2" t="s">
         <v>31</v>
       </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A12">
-        <v>2</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="A12" s="2">
+        <v>2</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="2" t="s">
         <v>34</v>
       </c>
+      <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A13">
-        <v>2</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="A13" s="2">
+        <v>2</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="2" t="s">
         <v>36</v>
       </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A14">
-        <v>2</v>
-      </c>
-      <c r="B14" t="s">
+      <c r="A14" s="2">
+        <v>2</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="2" t="s">
         <v>39</v>
       </c>
+      <c r="E14" s="2"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A15">
+      <c r="A15" s="2">
         <v>1</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="2" t="s">
         <v>41</v>
       </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A16">
+      <c r="A16" s="2">
         <v>1</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="2" t="s">
         <v>43</v>
       </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A17">
+      <c r="A17" s="2">
         <v>0</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="2" t="s">
         <v>46</v>
       </c>
+      <c r="E17" s="2"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A18">
+      <c r="A18" s="2">
         <v>0</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E18" t="s">
+      <c r="D18" s="2"/>
+      <c r="E18" s="2" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A19">
+      <c r="A19" s="2">
         <v>0</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="2" t="s">
         <v>51</v>
       </c>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A20">
+      <c r="A20" s="2">
         <v>0</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="2" t="s">
         <v>53</v>
       </c>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A21">
+      <c r="A21" s="2">
         <v>0</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="2" t="s">
         <v>55</v>
       </c>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A22">
+      <c r="A22" s="2">
         <v>0</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="2" t="s">
         <v>58</v>
       </c>
+      <c r="E22" s="2"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A23">
+      <c r="A23" s="2">
         <v>0</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="2" t="s">
         <v>60</v>
       </c>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A24">
+      <c r="A24" s="2">
         <v>0</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="2" t="s">
         <v>62</v>
       </c>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A25">
+      <c r="A25" s="2">
         <v>0</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="2" t="s">
         <v>64</v>
       </c>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.15">
-      <c r="A26">
+      <c r="A26" s="2">
         <v>0</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A27" s="2">
+        <v>2</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>67</v>
       </c>
+      <c r="C27" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A28" s="2">
+        <v>2</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A29" s="2">
+        <v>2</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A30" s="2">
+        <v>2</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A31" s="2">
+        <v>2</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A32" s="2">
+        <v>2</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A33" s="2">
+        <v>2</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A34" s="2">
+        <v>2</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A35" s="2">
+        <v>2</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A36" s="2">
+        <v>2</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A37" s="2">
+        <v>2</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A38" s="2">
+        <v>2</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A39" s="2">
+        <v>2</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A40" s="2">
+        <v>2</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A41" s="2">
+        <v>2</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A42" s="2">
+        <v>2</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="A43" s="2">
+        <v>2</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -948,7 +1354,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData/>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -958,7 +1364,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <sheetData/>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>